<commit_message>
Deterministic A16 bootstrap seeds; A17 design table
- code/A16retrainterm.py: the per-level bootstrap seed is derived from
  (target, m) with CRC-32, so tables a and b are a deterministic function
  of outputs/A16retrainterm_raw.json. outputs/A16retrainterm.xlsx and
  outputs/A16retrainterm_raw.json are the results of the rerun.
- code/A17designtable.py, outputs/A17designtable.xlsx: the replicate
  design table (3/5/10/21) and the single-face SD, computed from the
  stored variance components.
- paper/: recompiled manuscript and supplement.
- README.md: script and workbook counts, the derived quantities that are
  exported, and the precision of the five-face ceiling interval.
- docs/claim_evidence_map.md: C1.2, C1.5, C6.1 and C6.9-C6.11 follow the
  new workbooks; audit trail row 21.
</commit_message>
<xml_diff>
--- a/outputs/A16retrainterm.xlsx
+++ b/outputs/A16retrainterm.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表a逐m两臂" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表b合并与CI" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表c读法与限度" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表d重训臂对A9逐档" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,7 +484,17 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>两臂相对偏差之差(百分点)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>成分数中位(重训/固定)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Δ 自助种子</t>
         </is>
       </c>
     </row>
@@ -497,33 +508,39 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.542729</v>
+        <v>0.542728</v>
       </c>
       <c r="D2" t="n">
-        <v>0.533589</v>
+        <v>0.533567</v>
       </c>
       <c r="E2" t="n">
-        <v>0.537485</v>
+        <v>0.537442</v>
       </c>
       <c r="F2" t="n">
-        <v>0.003896</v>
+        <v>0.003875</v>
       </c>
       <c r="G2" t="n">
-        <v>0.003235</v>
+        <v>0.003198</v>
       </c>
       <c r="H2" t="n">
         <v>0.00457</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.966</v>
+        <v>-0.973936</v>
       </c>
       <c r="J2" t="n">
-        <v>-1.684</v>
-      </c>
-      <c r="K2" t="inlineStr">
+        <v>-1.687963</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.714027</v>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>20/24</t>
         </is>
+      </c>
+      <c r="M2" t="n">
+        <v>3753409266</v>
       </c>
     </row>
     <row r="3">
@@ -539,30 +556,36 @@
         <v>0.655233</v>
       </c>
       <c r="D3" t="n">
-        <v>0.646933</v>
+        <v>0.647045</v>
       </c>
       <c r="E3" t="n">
-        <v>0.649421</v>
+        <v>0.6493640000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>0.002487</v>
+        <v>0.002319</v>
       </c>
       <c r="G3" t="n">
-        <v>0.002032</v>
+        <v>0.001865</v>
       </c>
       <c r="H3" t="n">
-        <v>0.002977</v>
+        <v>0.002881</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.887</v>
+        <v>-0.895656</v>
       </c>
       <c r="J3" t="n">
-        <v>-1.267</v>
-      </c>
-      <c r="K3" t="inlineStr">
+        <v>-1.249535</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.353879</v>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>22/24</t>
         </is>
+      </c>
+      <c r="M3" t="n">
+        <v>1186016072</v>
       </c>
     </row>
     <row r="4">
@@ -578,30 +601,36 @@
         <v>0.703869</v>
       </c>
       <c r="D4" t="n">
-        <v>0.696222</v>
+        <v>0.696281</v>
       </c>
       <c r="E4" t="n">
-        <v>0.698007</v>
+        <v>0.697944</v>
       </c>
       <c r="F4" t="n">
-        <v>0.001785</v>
+        <v>0.001663</v>
       </c>
       <c r="G4" t="n">
-        <v>0.001428</v>
+        <v>0.001306</v>
       </c>
       <c r="H4" t="n">
-        <v>0.002159</v>
+        <v>0.002109</v>
       </c>
       <c r="I4" t="n">
-        <v>-0.833</v>
+        <v>-0.841761</v>
       </c>
       <c r="J4" t="n">
-        <v>-1.086</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>23/24</t>
-        </is>
+        <v>-1.078075</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.236313</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>22/24</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>834018270</v>
       </c>
     </row>
     <row r="5">
@@ -617,30 +646,36 @@
         <v>0.730999</v>
       </c>
       <c r="D5" t="n">
-        <v>0.723841</v>
+        <v>0.723782</v>
       </c>
       <c r="E5" t="n">
-        <v>0.725189</v>
+        <v>0.725122</v>
       </c>
       <c r="F5" t="n">
-        <v>0.001347</v>
+        <v>0.00134</v>
       </c>
       <c r="G5" t="n">
-        <v>0.001098</v>
+        <v>0.000968</v>
       </c>
       <c r="H5" t="n">
-        <v>0.001622</v>
+        <v>0.001768</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.795</v>
+        <v>-0.803935</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.979</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>24/24</t>
-        </is>
+        <v>-0.987187</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.183251</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>22/24</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>2949811837</v>
       </c>
     </row>
     <row r="6">
@@ -653,33 +688,39 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.748305</v>
+        <v>0.748304</v>
       </c>
       <c r="D6" t="n">
-        <v>0.741417</v>
+        <v>0.741439</v>
       </c>
       <c r="E6" t="n">
-        <v>0.742568</v>
+        <v>0.742499</v>
       </c>
       <c r="F6" t="n">
-        <v>0.001151</v>
+        <v>0.00106</v>
       </c>
       <c r="G6" t="n">
-        <v>0.000977</v>
+        <v>0.000738</v>
       </c>
       <c r="H6" t="n">
-        <v>0.001367</v>
+        <v>0.001381</v>
       </c>
       <c r="I6" t="n">
-        <v>-0.767</v>
+        <v>-0.775819</v>
       </c>
       <c r="J6" t="n">
-        <v>-0.921</v>
-      </c>
-      <c r="K6" t="inlineStr">
+        <v>-0.917489</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.14167</v>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M6" t="n">
+        <v>3637886699</v>
       </c>
     </row>
     <row r="7">
@@ -695,30 +736,36 @@
         <v>0.760304</v>
       </c>
       <c r="D7" t="n">
-        <v>0.753745</v>
+        <v>0.7536620000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>0.754643</v>
+        <v>0.754572</v>
       </c>
       <c r="F7" t="n">
-        <v>0.000898</v>
+        <v>0.00091</v>
       </c>
       <c r="G7" t="n">
-        <v>0.000736</v>
+        <v>0.000623</v>
       </c>
       <c r="H7" t="n">
-        <v>0.00106</v>
+        <v>0.001241</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.745</v>
+        <v>-0.753951</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.863</v>
-      </c>
-      <c r="K7" t="inlineStr">
+        <v>-0.873604</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.119653</v>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M7" t="n">
+        <v>1104998225</v>
       </c>
     </row>
     <row r="8">
@@ -731,33 +778,39 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.769114</v>
+        <v>0.769113</v>
       </c>
       <c r="D8" t="n">
-        <v>0.762747</v>
+        <v>0.762651</v>
       </c>
       <c r="E8" t="n">
-        <v>0.763522</v>
+        <v>0.76345</v>
       </c>
       <c r="F8" t="n">
-        <v>0.000775</v>
+        <v>0.000799</v>
       </c>
       <c r="G8" t="n">
-        <v>0.000614</v>
+        <v>0.0005509999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>0.000929</v>
+        <v>0.001109</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.727</v>
+        <v>-0.7363499999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.828</v>
-      </c>
-      <c r="K8" t="inlineStr">
+        <v>-0.840259</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.103909</v>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M8" t="n">
+        <v>920379335</v>
       </c>
     </row>
     <row r="9">
@@ -773,30 +826,36 @@
         <v>0.775856</v>
       </c>
       <c r="D9" t="n">
-        <v>0.769637</v>
+        <v>0.769571</v>
       </c>
       <c r="E9" t="n">
-        <v>0.770329</v>
+        <v>0.7702560000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>0.000692</v>
+        <v>0.000684</v>
       </c>
       <c r="G9" t="n">
-        <v>0.000519</v>
+        <v>0.000383</v>
       </c>
       <c r="H9" t="n">
-        <v>0.000873</v>
+        <v>0.000993</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.712</v>
+        <v>-0.721803</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.802</v>
-      </c>
-      <c r="K9" t="inlineStr">
+        <v>-0.810007</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.088204</v>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M9" t="n">
+        <v>2791621206</v>
       </c>
     </row>
     <row r="10">
@@ -812,30 +871,36 @@
         <v>0.781182</v>
       </c>
       <c r="D10" t="n">
-        <v>0.775093</v>
+        <v>0.775025</v>
       </c>
       <c r="E10" t="n">
-        <v>0.775714</v>
+        <v>0.775639</v>
       </c>
       <c r="F10" t="n">
-        <v>0.000621</v>
+        <v>0.000614</v>
       </c>
       <c r="G10" t="n">
-        <v>0.00045</v>
+        <v>0.000343</v>
       </c>
       <c r="H10" t="n">
-        <v>0.000791</v>
+        <v>0.000889</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.7</v>
+        <v>-0.709527</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.78</v>
-      </c>
-      <c r="K10" t="inlineStr">
+        <v>-0.788127</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.0786</v>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M10" t="n">
+        <v>3512988352</v>
       </c>
     </row>
     <row r="11">
@@ -851,30 +916,36 @@
         <v>0.785496</v>
       </c>
       <c r="D11" t="n">
-        <v>0.779518</v>
+        <v>0.7795029999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>0.78008</v>
+        <v>0.7800049999999999</v>
       </c>
       <c r="F11" t="n">
-        <v>0.000562</v>
+        <v>0.000503</v>
       </c>
       <c r="G11" t="n">
-        <v>0.000399</v>
+        <v>0.000323</v>
       </c>
       <c r="H11" t="n">
-        <v>0.000725</v>
+        <v>0.000681</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.6989919999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.761</v>
-      </c>
-      <c r="K11" t="inlineStr">
+        <v>-0.762972</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.06397899999999999</v>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M11" t="n">
+        <v>2813850731</v>
       </c>
     </row>
     <row r="12">
@@ -890,30 +961,36 @@
         <v>0.796811</v>
       </c>
       <c r="D12" t="n">
-        <v>0.791224</v>
+        <v>0.791164</v>
       </c>
       <c r="E12" t="n">
-        <v>0.791564</v>
+        <v>0.7914870000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>0.00034</v>
+        <v>0.000323</v>
       </c>
       <c r="G12" t="n">
-        <v>0.000204</v>
+        <v>0.000149</v>
       </c>
       <c r="H12" t="n">
-        <v>0.000483</v>
+        <v>0.000497</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.659</v>
+        <v>-0.668156</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.701</v>
-      </c>
-      <c r="K12" t="inlineStr">
+        <v>-0.708692</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.040536</v>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M12" t="n">
+        <v>2698653810</v>
       </c>
     </row>
     <row r="13">
@@ -926,33 +1003,39 @@
         <v>20</v>
       </c>
       <c r="C13" t="n">
-        <v>0.805514</v>
+        <v>0.805513</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8002010000000001</v>
+        <v>0.800157</v>
       </c>
       <c r="E13" t="n">
-        <v>0.800437</v>
+        <v>0.800359</v>
       </c>
       <c r="F13" t="n">
-        <v>0.000236</v>
+        <v>0.000202</v>
       </c>
       <c r="G13" t="n">
-        <v>0.000116</v>
+        <v>3.4e-05</v>
       </c>
       <c r="H13" t="n">
-        <v>0.000349</v>
+        <v>0.000369</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.63</v>
+        <v>-0.639951</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.66</v>
-      </c>
-      <c r="K13" t="inlineStr">
+        <v>-0.66497</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.025019</v>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M13" t="n">
+        <v>2358945704</v>
       </c>
     </row>
     <row r="14">
@@ -990,10 +1073,16 @@
       <c r="J14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M14" t="n">
+        <v>2831108708</v>
       </c>
     </row>
     <row r="15">
@@ -1024,15 +1113,21 @@
         <v>0.004339</v>
       </c>
       <c r="I15" t="n">
-        <v>-0.92</v>
+        <v>-0.9202979999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>-1.584</v>
-      </c>
-      <c r="K15" t="inlineStr">
+        <v>-1.583879</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.663581</v>
+      </c>
+      <c r="L15" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M15" t="n">
+        <v>1086880583</v>
       </c>
     </row>
     <row r="16">
@@ -1057,21 +1152,27 @@
         <v>0.002213</v>
       </c>
       <c r="G16" t="n">
-        <v>0.001814</v>
+        <v>0.001836</v>
       </c>
       <c r="H16" t="n">
-        <v>0.002641</v>
+        <v>0.002612</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.593</v>
+        <v>-0.592549</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.917</v>
-      </c>
-      <c r="K16" t="inlineStr">
+        <v>-0.916741</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.324191</v>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M16" t="n">
+        <v>3653315325</v>
       </c>
     </row>
     <row r="17">
@@ -1096,21 +1197,27 @@
         <v>0.00156</v>
       </c>
       <c r="G17" t="n">
-        <v>0.00126</v>
+        <v>0.001243</v>
       </c>
       <c r="H17" t="n">
-        <v>0.001919</v>
+        <v>0.001886</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.439</v>
+        <v>-0.439201</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.652</v>
-      </c>
-      <c r="K17" t="inlineStr">
+        <v>-0.651958</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.212757</v>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M17" t="n">
+        <v>2932218475</v>
       </c>
     </row>
     <row r="18">
@@ -1138,18 +1245,24 @@
         <v>0.000944</v>
       </c>
       <c r="H18" t="n">
-        <v>0.001501</v>
+        <v>0.001499</v>
       </c>
       <c r="I18" t="n">
-        <v>-0.351</v>
+        <v>-0.350538</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.508</v>
-      </c>
-      <c r="K18" t="inlineStr">
+        <v>-0.508055</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.157517</v>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M18" t="n">
+        <v>815960008</v>
       </c>
     </row>
     <row r="19">
@@ -1180,15 +1293,21 @@
         <v>0.001237</v>
       </c>
       <c r="I19" t="n">
-        <v>-0.293</v>
+        <v>-0.292719</v>
       </c>
       <c r="J19" t="n">
-        <v>-0.417</v>
-      </c>
-      <c r="K19" t="inlineStr">
+        <v>-0.417309</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.12459</v>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M19" t="n">
+        <v>1202044766</v>
       </c>
     </row>
     <row r="20">
@@ -1216,18 +1335,24 @@
         <v>0.000615</v>
       </c>
       <c r="H20" t="n">
-        <v>0.001037</v>
+        <v>0.001052</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.252</v>
+        <v>-0.251999</v>
       </c>
       <c r="J20" t="n">
-        <v>-0.355</v>
-      </c>
-      <c r="K20" t="inlineStr">
+        <v>-0.354758</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.102759</v>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M20" t="n">
+        <v>3735875300</v>
       </c>
     </row>
     <row r="21">
@@ -1258,15 +1383,21 @@
         <v>0.000904</v>
       </c>
       <c r="I21" t="n">
-        <v>-0.222</v>
+        <v>-0.221748</v>
       </c>
       <c r="J21" t="n">
-        <v>-0.309</v>
-      </c>
-      <c r="K21" t="inlineStr">
+        <v>-0.30899</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.087242</v>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M21" t="n">
+        <v>2846613106</v>
       </c>
     </row>
     <row r="22">
@@ -1297,15 +1428,21 @@
         <v>0.000812</v>
       </c>
       <c r="I22" t="n">
-        <v>-0.198</v>
+        <v>-0.198373</v>
       </c>
       <c r="J22" t="n">
-        <v>-0.274</v>
-      </c>
-      <c r="K22" t="inlineStr">
+        <v>-0.27403</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.075657</v>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M22" t="n">
+        <v>957662179</v>
       </c>
     </row>
     <row r="23">
@@ -1336,15 +1473,21 @@
         <v>0.000729</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.18</v>
+        <v>-0.179761</v>
       </c>
       <c r="J23" t="n">
-        <v>-0.246</v>
-      </c>
-      <c r="K23" t="inlineStr">
+        <v>-0.246443</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.06668300000000001</v>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M23" t="n">
+        <v>1309930357</v>
       </c>
     </row>
     <row r="24">
@@ -1372,18 +1515,24 @@
         <v>0.000341</v>
       </c>
       <c r="H24" t="n">
-        <v>0.000655</v>
+        <v>0.000662</v>
       </c>
       <c r="I24" t="n">
-        <v>-0.165</v>
+        <v>-0.164583</v>
       </c>
       <c r="J24" t="n">
-        <v>-0.224</v>
-      </c>
-      <c r="K24" t="inlineStr">
+        <v>-0.224115</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.059532</v>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M24" t="n">
+        <v>472105833</v>
       </c>
     </row>
     <row r="25">
@@ -1408,21 +1557,27 @@
         <v>0.000343</v>
       </c>
       <c r="G25" t="n">
-        <v>0.000224</v>
+        <v>0.000228</v>
       </c>
       <c r="H25" t="n">
         <v>0.000482</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.124</v>
+        <v>-0.124279</v>
       </c>
       <c r="J25" t="n">
-        <v>-0.166</v>
-      </c>
-      <c r="K25" t="inlineStr">
+        <v>-0.16557</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.041292</v>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M25" t="n">
+        <v>458098544</v>
       </c>
     </row>
     <row r="26">
@@ -1450,18 +1605,24 @@
         <v>0.000137</v>
       </c>
       <c r="H26" t="n">
-        <v>0.000348</v>
+        <v>0.000349</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.093</v>
+        <v>-0.092685</v>
       </c>
       <c r="J26" t="n">
-        <v>-0.121</v>
-      </c>
-      <c r="K26" t="inlineStr">
+        <v>-0.120502</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.027817</v>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M26" t="n">
+        <v>923701418</v>
       </c>
     </row>
     <row r="27">
@@ -1499,10 +1660,16 @@
       <c r="J27" t="n">
         <v>0</v>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>24/24</t>
         </is>
+      </c>
+      <c r="M27" t="n">
+        <v>936332241</v>
       </c>
     </row>
   </sheetData>
@@ -1566,18 +1733,18 @@
         <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>0.001233</v>
+        <v>0.001191</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[0.000976, 0.001512]</t>
+          <t>[0.000929, 0.001472]</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-0.736</v>
+        <v>-0.745151</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.845</v>
+        <v>-0.856931</v>
       </c>
       <c r="G2" t="n">
         <v>12</v>
@@ -1601,10 +1768,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-0.237</v>
+        <v>-0.236873</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.332</v>
+        <v>-0.331874</v>
       </c>
       <c r="G3" t="n">
         <v>12</v>
@@ -1621,7 +1788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,32 +1835,618 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Δ = R²_固定 − R²_重训 &gt; 0 表示重训在带噪标签上损失了性能，即式 (degrade) 作为重训过程的预言偏乐观、作为设计规则的下限方向保守。CI 由与 A9 相同的两级簇自助给出（2000 次，按单元重抽）。</t>
+          <t>Δ = R²_固定 − R²_重训 &gt; 0 表示重训在带噪标签上损失了性能，即式 (degrade) 作为重训过程的预言偏乐观、作为设计规则的下限方向保守。CI 由与 A9 相同的两级簇自助给出（2000 次，按单元重抽）。逐档 CI 的种子由 (目标, m) 经 CRC-32 得出（表a「Δ 自助种子」列），合并 CI 的种子为 7，两者都与进程和平台无关，表a、表b 因而是 A16retrainterm_raw.json 的确定性函数。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>平台效应为何不污染 Δ</t>
+          <t>跨平台</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>本机重训臂与 A9 已发布的逐次值并非逐位相同：实测同一 (DM, m=5, 20060515) 单元6 次重复中 1 次逐位相同、其余 R² 差 ~1e-3，机制是内层 CV 的 MSE 曲线在高成分数段近平坦，BLAS 浮点差翻转了所选成分数（A9 记录 22/22/22/24/24/24，本机 24/24/24/22/24/22）。这不影响本表：两条臂在**同一台机器、同一次重复、同一份噪声、同一划分**上跑，Δ 是配对差，平台效应对两臂同向作用后相消。因此 Δ 可跨平台读，而两臂各自的绝对 R² 只在本机口径下成立。</t>
+          <t>本次运行的重训臂与 A9 已发布值逐项比对：逐次 R² 在 780 次重复中 442 次逐位相同，192 次所选成分数不同，最大差 1.86e-03；逐档相对偏差与 A9 至多差 0.0133 个百分点（DM，m=1，见表d）。机制是内层 CV 的 MSE 曲线在高成分数段近平坦，BLAS 浮点差可翻转所选成分数，翻转移动的是该次重复的 R²。两条臂在同一台机器、同一次重复、同一份噪声、同一划分上跑，Δ 是同次配对差；翻转可以只落在一条臂上，所以 Δ 与两臂各自的绝对 R² 一样，都是单一平台下的值。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>运行环境</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Python 3.10.20，numpy 2.2.6，scipy 1.15.3，scikit-learn 1.6.1，pandas 2.3.3；BLAS scipy-openblas 0.3.29；Linux x86_64，CPU AMD EPYC 7502 32-Core Processor。整轮重跑的逐位复现以同一平台、同一 BLAS 为前提。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>限度（必须一并读）</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>① 固定臂仍用同一训练集拟合，只是标签干净，因此它是『注入前固定』的一个实现而非唯一实现；② 本表不构成对不变性的证明，只给出该假设在本数据、本评估器下留下的差额；③ 本脚本不改 A9 的任何预注册判据，A9 产物未被覆盖。</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>目标</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>A9 相对偏差(%)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>本次重训臂相对偏差(%)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>差(百分点)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>差的绝对值(全精度)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-1.674658</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-1.687963</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.013304</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.01330446728046164</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-1.255371</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-1.249535</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.005836</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.005835857576408365</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-1.075855</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-1.078075</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.00222</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.002219528812930083</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.982398</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.987187</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.004788</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.004788077874273711</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-0.923037</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.917489</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.005547</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.005547376911241297</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-0.876443</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-0.873604</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.002839</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.002839394684817087</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-0.844415</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-0.840259</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.004157</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.004156677738020864</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-0.817295</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-0.810007</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.007288</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.00728798284984622</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-0.795189</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-0.788127</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.007062</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.007062038543992344</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-0.768709</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-0.762972</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.005737</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.005737253860249591</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>14</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-0.7158409999999999</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-0.708692</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.007149</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.007148843188953258</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>20</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-0.670517</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-0.66497</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.005547</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.005546756713892265</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-1.585091</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-1.583879</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.001211</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.001211434120773625</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-0.916741</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-0.916741</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-0.651958</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.651958</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.220446049250313e-14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-0.508055</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-0.508055</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>-0.417309</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-0.417309</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-0.354758</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-0.354758</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-0.30899</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.30899</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3.33066907387547e-14</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-0.27403</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-0.27403</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1.110223024625157e-14</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>9</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-0.246443</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-0.246443</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" t="n">
+        <v>-0.224115</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-0.224115</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>14</v>
+      </c>
+      <c r="C24" t="n">
+        <v>-0.16557</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-0.16557</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2.220446049250313e-14</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SSC</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>20</v>
+      </c>
+      <c r="C25" t="n">
+        <v>-0.120502</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.120502</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1.110223024625157e-14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>